<commit_message>
Ensure age consistency in social care
The UKHLS appears to allow caregiving from age 16, but the simulation was restricted to 18+.
</commit_message>
<xml_diff>
--- a/documentation/SimPaths Stata Parameters.xlsx
+++ b/documentation/SimPaths Stata Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9BFC8D-9522-3A4E-B984-CC84A75C3949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76D75FB1-39BD-934E-AC89-206342B8C055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17840" xr2:uid="{63B995B5-DCE1-5E4F-9426-71F242651852}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17800" xr2:uid="{63B995B5-DCE1-5E4F-9426-71F242651852}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
   <si>
     <t>Parameters in SimPaths</t>
   </si>
@@ -186,6 +186,9 @@
   </si>
   <si>
     <t>365.25/7</t>
+  </si>
+  <si>
+    <t>MIN_AGE_TO_PROVIDE_CARE</t>
   </si>
 </sst>
 </file>
@@ -256,7 +259,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -520,11 +523,57 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -631,14 +680,17 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -974,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8738A44-8083-4443-A4E7-DCC9B2B5EE0F}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31" style="11" customWidth="1"/>
@@ -1189,13 +1241,13 @@
       <c r="A15" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="38">
+      <c r="B15" s="21">
         <v>49</v>
       </c>
-      <c r="C15" s="39" t="s">
+      <c r="C15" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="40">
+      <c r="D15" s="18">
         <v>49</v>
       </c>
       <c r="E15" s="22" t="s">
@@ -1258,51 +1310,62 @@
       </c>
       <c r="E19" s="22"/>
     </row>
-    <row r="20" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="23" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="38"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" s="40">
+        <v>16</v>
+      </c>
+      <c r="E20" s="41"/>
+    </row>
+    <row r="21" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="24">
+      <c r="B21" s="24">
         <v>75</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C21" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="25">
+      <c r="D21" s="25">
         <v>75</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E21" s="26" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="10" t="s">
+    <row r="23" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="27"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24" s="18">
-        <v>79</v>
-      </c>
+      <c r="B24" s="27"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="18">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="18">
+      <c r="B26" s="18">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+    <row r="27" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="25">
+      <c r="B27" s="25">
         <v>17</v>
       </c>
     </row>

</xml_diff>